<commit_message>
feat: add initial payment + cadastre handover plan for 22, 25, 34, 39 m2 units
</commit_message>
<xml_diff>
--- a/Янги Куйлик -2 лойихаси нархлари.xlsx
+++ b/Янги Куйлик -2 лойихаси нархлари.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="31">
   <si>
     <t xml:space="preserve">1-хоналига 29 млн., 2-хоналига 39 млн, 3-хоналига 69 млн сум тулаб уй харид килганга уйлар нархи </t>
   </si>
@@ -108,6 +108,18 @@
   </si>
   <si>
     <t>4-тўлов тури</t>
+  </si>
+  <si>
+    <t>Бошланғич тўлов суммаси (сўм)</t>
+  </si>
+  <si>
+    <t>Қолдиқ кадастр вакти тўланади (2-3-4-қаватларда) (сўм)</t>
+  </si>
+  <si>
+    <t>Қолдиқ кадастр вакти тўланади  (5-6-7-8-қаватларда) (сўм)</t>
+  </si>
+  <si>
+    <t>Қолдиқ кадастр вакти тўланади  (9-10-11-12-қаватларда) (сўм)</t>
   </si>
 </sst>
 </file>
@@ -812,7 +824,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -841,6 +853,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1376,7 +1397,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S50"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr defaultColWidth="15" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
@@ -1513,15 +1534,15 @@
         <v>120000000</v>
       </c>
       <c r="O3" s="8">
-        <f>H3-K3-N3</f>
+        <f t="shared" ref="O3:O8" si="0">H3-K3-N3</f>
         <v>312250000</v>
       </c>
       <c r="P3" s="8">
-        <f>I3-K3-N3</f>
+        <f t="shared" ref="P3:P8" si="1">I3-K3-N3</f>
         <v>291750000</v>
       </c>
       <c r="Q3" s="8">
-        <f>J3-K3-N3</f>
+        <f t="shared" ref="Q3:Q8" si="2">J3-K3-N3</f>
         <v>271250000</v>
       </c>
     </row>
@@ -1567,15 +1588,15 @@
         <v>120000000</v>
       </c>
       <c r="O4" s="8">
-        <f>H4-K4-N4</f>
+        <f t="shared" si="0"/>
         <v>334750000</v>
       </c>
       <c r="P4" s="8">
-        <f>I4-K4-N4</f>
+        <f t="shared" si="1"/>
         <v>313250000</v>
       </c>
       <c r="Q4" s="8">
-        <f>J4-K4-N4</f>
+        <f t="shared" si="2"/>
         <v>291750000</v>
       </c>
     </row>
@@ -1621,15 +1642,15 @@
         <v>150000000</v>
       </c>
       <c r="O5" s="8">
-        <f>H5-K5-N5</f>
+        <f t="shared" si="0"/>
         <v>391500000</v>
       </c>
       <c r="P5" s="8">
-        <f>I5-K5-N5</f>
+        <f t="shared" si="1"/>
         <v>364500000</v>
       </c>
       <c r="Q5" s="8">
-        <f>J5-K5-N5</f>
+        <f t="shared" si="2"/>
         <v>337500000</v>
       </c>
     </row>
@@ -1675,15 +1696,15 @@
         <v>150000000</v>
       </c>
       <c r="O6" s="8">
-        <f>H6-K6-N6</f>
+        <f t="shared" si="0"/>
         <v>402250000</v>
       </c>
       <c r="P6" s="8">
-        <f>I6-K6-N6</f>
+        <f t="shared" si="1"/>
         <v>374750000</v>
       </c>
       <c r="Q6" s="8">
-        <f>J6-K6-N6</f>
+        <f t="shared" si="2"/>
         <v>347250000</v>
       </c>
     </row>
@@ -1729,15 +1750,15 @@
         <v>180000000</v>
       </c>
       <c r="O7" s="8">
-        <f>H7-K7-N7</f>
+        <f t="shared" si="0"/>
         <v>468500000</v>
       </c>
       <c r="P7" s="8">
-        <f>I7-K7-N7</f>
+        <f t="shared" si="1"/>
         <v>433500000</v>
       </c>
       <c r="Q7" s="8">
-        <f>J7-K7-N7</f>
+        <f t="shared" si="2"/>
         <v>398500000</v>
       </c>
     </row>
@@ -1783,15 +1804,15 @@
         <v>180000000</v>
       </c>
       <c r="O8" s="8">
-        <f>H8-K8-N8</f>
+        <f t="shared" si="0"/>
         <v>540250000</v>
       </c>
       <c r="P8" s="8">
-        <f>I8-K8-N8</f>
+        <f t="shared" si="1"/>
         <v>501750000</v>
       </c>
       <c r="Q8" s="8">
-        <f>J8-K8-N8</f>
+        <f t="shared" si="2"/>
         <v>463250000</v>
       </c>
     </row>
@@ -2758,20 +2779,24 @@
       </c>
     </row>
     <row r="39" spans="1:19">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="J39" s="4"/>
-    </row>
-    <row r="40" ht="45" spans="1:19">
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+    </row>
+    <row r="40" ht="75" spans="1:19">
       <c r="A40" s="6" t="s">
         <v>26</v>
       </c>
@@ -2801,6 +2826,18 @@
       </c>
       <c r="J40" s="6" t="s">
         <v>10</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M40" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:19">
@@ -2821,7 +2858,7 @@
         <v>7202500</v>
       </c>
       <c r="G41" s="8">
-        <v>6867500</v>
+        <v>6662500</v>
       </c>
       <c r="H41" s="8">
         <v>165825000</v>
@@ -2830,7 +2867,23 @@
         <v>158455000</v>
       </c>
       <c r="J41" s="8">
-        <v>151085000</v>
+        <f>C41*G41</f>
+        <v>146575000</v>
+      </c>
+      <c r="K41" s="11">
+        <v>146575000</v>
+      </c>
+      <c r="L41" s="12">
+        <f>H41-K41</f>
+        <v>19250000</v>
+      </c>
+      <c r="M41" s="12">
+        <f>I41-K41</f>
+        <v>11880000</v>
+      </c>
+      <c r="N41" s="12">
+        <f>J41-K41</f>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:19">
@@ -2862,6 +2915,21 @@
       <c r="J42" s="8">
         <v>171687500</v>
       </c>
+      <c r="K42" s="11">
+        <v>146575000</v>
+      </c>
+      <c r="L42" s="12">
+        <f>H42-K42</f>
+        <v>41862500</v>
+      </c>
+      <c r="M42" s="12">
+        <f>I42-K42</f>
+        <v>33487500</v>
+      </c>
+      <c r="N42" s="12">
+        <f>J42-K42</f>
+        <v>25112500</v>
+      </c>
     </row>
     <row r="43" spans="1:19">
       <c r="A43" s="6"/>
@@ -2892,6 +2960,21 @@
       <c r="J43" s="8">
         <v>233495000</v>
       </c>
+      <c r="K43" s="11">
+        <v>177000000</v>
+      </c>
+      <c r="L43" s="12">
+        <f>H43-K43</f>
+        <v>79275000</v>
+      </c>
+      <c r="M43" s="12">
+        <f>I43-K43</f>
+        <v>67885000</v>
+      </c>
+      <c r="N43" s="12">
+        <f>J43-K43</f>
+        <v>56495000</v>
+      </c>
     </row>
     <row r="44" spans="1:19">
       <c r="A44" s="6"/>
@@ -2899,7 +2982,7 @@
         <v>4</v>
       </c>
       <c r="C44" s="6">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D44" s="6">
         <v>1</v>
@@ -2921,6 +3004,21 @@
       </c>
       <c r="J44" s="8">
         <v>281567500</v>
+      </c>
+      <c r="K44" s="11">
+        <v>177000000</v>
+      </c>
+      <c r="L44" s="12">
+        <f>H44-K44</f>
+        <v>132037500</v>
+      </c>
+      <c r="M44" s="12">
+        <f>I44-K44</f>
+        <v>118302500</v>
+      </c>
+      <c r="N44" s="12">
+        <f>J44-K44</f>
+        <v>104567500</v>
       </c>
     </row>
     <row r="45" spans="1:19">
@@ -2929,7 +3027,7 @@
         <v>5</v>
       </c>
       <c r="C45" s="6">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D45" s="6">
         <v>1</v>
@@ -2959,7 +3057,7 @@
         <v>6</v>
       </c>
       <c r="C46" s="6">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D46" s="6">
         <v>1</v>
@@ -2974,13 +3072,13 @@
         <v>6867500</v>
       </c>
       <c r="H46" s="8">
-        <v>369337500</v>
+        <v>293962500</v>
       </c>
       <c r="I46" s="8">
-        <v>352922500</v>
+        <v>280897500</v>
       </c>
       <c r="J46" s="8">
-        <v>336507500</v>
+        <v>267832500</v>
       </c>
     </row>
     <row r="47" spans="1:19">
@@ -2989,28 +3087,28 @@
         <v>7</v>
       </c>
       <c r="C47" s="6">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D47" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" s="8">
+        <v>7537500</v>
+      </c>
+      <c r="F47" s="8">
         <v>7202500</v>
       </c>
-      <c r="F47" s="8">
+      <c r="G47" s="8">
         <v>6867500</v>
       </c>
-      <c r="G47" s="8">
-        <v>6532500</v>
-      </c>
       <c r="H47" s="8">
-        <v>388935000</v>
+        <v>369337500</v>
       </c>
       <c r="I47" s="8">
-        <v>370845000</v>
+        <v>352922500</v>
       </c>
       <c r="J47" s="8">
-        <v>352755000</v>
+        <v>336507500</v>
       </c>
     </row>
     <row r="48" spans="1:19">
@@ -3019,7 +3117,7 @@
         <v>8</v>
       </c>
       <c r="C48" s="6">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D48" s="6">
         <v>2</v>
@@ -3034,13 +3132,13 @@
         <v>6532500</v>
       </c>
       <c r="H48" s="8">
-        <v>396137500</v>
+        <v>388935000</v>
       </c>
       <c r="I48" s="8">
-        <v>377712500</v>
+        <v>370845000</v>
       </c>
       <c r="J48" s="8">
-        <v>359287500</v>
+        <v>352755000</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -3049,28 +3147,28 @@
         <v>9</v>
       </c>
       <c r="C49" s="6">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D49" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E49" s="8">
+        <v>7202500</v>
+      </c>
+      <c r="F49" s="8">
         <v>6867500</v>
       </c>
-      <c r="F49" s="8">
+      <c r="G49" s="8">
         <v>6532500</v>
       </c>
-      <c r="G49" s="8">
-        <v>6197500</v>
-      </c>
       <c r="H49" s="8">
-        <v>480725000</v>
+        <v>396137500</v>
       </c>
       <c r="I49" s="8">
-        <v>457275000</v>
+        <v>377712500</v>
       </c>
       <c r="J49" s="8">
-        <v>433825000</v>
+        <v>359287500</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -3079,7 +3177,7 @@
         <v>10</v>
       </c>
       <c r="C50" s="6">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D50" s="6">
         <v>3</v>
@@ -3094,12 +3192,42 @@
         <v>6197500</v>
       </c>
       <c r="H50" s="8">
+        <v>480725000</v>
+      </c>
+      <c r="I50" s="8">
+        <v>457275000</v>
+      </c>
+      <c r="J50" s="8">
+        <v>433825000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
+      <c r="A51" s="6"/>
+      <c r="B51" s="6">
+        <v>11</v>
+      </c>
+      <c r="C51" s="6">
+        <v>77</v>
+      </c>
+      <c r="D51" s="6">
+        <v>3</v>
+      </c>
+      <c r="E51" s="8">
+        <v>6867500</v>
+      </c>
+      <c r="F51" s="8">
+        <v>6532500</v>
+      </c>
+      <c r="G51" s="8">
+        <v>6197500</v>
+      </c>
+      <c r="H51" s="8">
         <v>528797500</v>
       </c>
-      <c r="I50" s="8">
+      <c r="I51" s="8">
         <v>503002500</v>
       </c>
-      <c r="J50" s="8">
+      <c r="J51" s="8">
         <v>477207500</v>
       </c>
     </row>
@@ -3108,11 +3236,11 @@
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A13:S13"/>
     <mergeCell ref="A26:S26"/>
-    <mergeCell ref="A39:J39"/>
+    <mergeCell ref="A39:N39"/>
     <mergeCell ref="A2:A8"/>
     <mergeCell ref="A14:A21"/>
     <mergeCell ref="A27:A34"/>
-    <mergeCell ref="A40:A50"/>
+    <mergeCell ref="A40:A51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>